<commit_message>
Tier 2 products launched
</commit_message>
<xml_diff>
--- a/Reyval products.xlsx
+++ b/Reyval products.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIDDHU\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIDDHU\Desktop\Reyval\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2D1B159-F3F1-4448-A04F-F40E2D8897DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71A2395-06F5-45AA-979E-8855AD8F71F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="tier 1 products" sheetId="1" r:id="rId1"/>
+    <sheet name="Tier 2 products" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="83">
   <si>
     <t>Category</t>
   </si>
@@ -211,6 +212,69 @@
   </si>
   <si>
     <t>Mens waist belt</t>
+  </si>
+  <si>
+    <t>https://www.meesho.com/urbane-ravishing-men-sweatshirts/p/76g1q9</t>
+  </si>
+  <si>
+    <t>Meesho</t>
+  </si>
+  <si>
+    <t>White Fasion Hoodie</t>
+  </si>
+  <si>
+    <t>Bat Man Theme Hoodie</t>
+  </si>
+  <si>
+    <t>https://www.meesho.com/men-printed-round-neck-sweatshirt-by-hip-hop-fashion/p/4y4mwi</t>
+  </si>
+  <si>
+    <t>https://www.meesho.com/men-sweatshirt-sweatshirt-for-men-winter-wear-warm-hoodie-green-hoodie/p/awi93m</t>
+  </si>
+  <si>
+    <t>https://www.meesho.com/keesor-men-sweatshirtmen-jacketmen-cotton-hooded-neck-sweatshirt/p/7q1nam</t>
+  </si>
+  <si>
+    <t>Mens Stylish Green Hoodie</t>
+  </si>
+  <si>
+    <t>Mens Trendy Sweat Shirt</t>
+  </si>
+  <si>
+    <t>https://www.meesho.com/men-regular-fit-formal-stretchable-with-expandable-waist-light-gray-pant/p/9h1nf4</t>
+  </si>
+  <si>
+    <t>Mens grey formal pant</t>
+  </si>
+  <si>
+    <t>https://www.meesho.com/men-slim-fit-ankle-length-black-best-premium-quality-low-price-formal-wear-trouser-or-pant/p/d10d9g</t>
+  </si>
+  <si>
+    <t>Black Business formal trousers</t>
+  </si>
+  <si>
+    <t>https://www.meesho.com/mens-formal-pants-for-men-mens-slimm-fit-formal-pant-non-stretchable-trouser-office-wear-trousers/p/abmain</t>
+  </si>
+  <si>
+    <t>https://www.meesho.com/men-printed-black-tranding-track-pants-fabric-cotton-pack-of-1/p/fjf39g</t>
+  </si>
+  <si>
+    <t>Mens formal Blue Pants</t>
+  </si>
+  <si>
+    <t>Mens street ware pants</t>
+  </si>
+  <si>
+    <t>https://www.meesho.com/kezual-black-oversized-track-pant-l-best-track-pant-for-street-wear-fashion-l-comfort-with-style/p/ff8aaq</t>
+  </si>
+  <si>
+    <t>Mens printed pants</t>
+  </si>
+  <si>
+    <t>https://www.meesho.com/shirt-for-men/p/8yk31j</t>
+  </si>
+  <si>
+    <t>Mens Texured Shirt</t>
   </si>
 </sst>
 </file>
@@ -257,7 +321,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -293,12 +357,132 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
@@ -312,6 +496,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1280,4 +1473,528 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId24"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9785A799-A3B0-435F-9C0F-A7FD7012CF10}">
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="35.44140625" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.44140625" customWidth="1"/>
+    <col min="5" max="5" width="17.77734375" customWidth="1"/>
+    <col min="6" max="7" width="17.88671875" customWidth="1"/>
+    <col min="8" max="8" width="131.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="7"/>
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="10">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1">
+        <v>353</v>
+      </c>
+      <c r="E2" s="1">
+        <v>453</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1999</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="10">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1">
+        <v>333</v>
+      </c>
+      <c r="E3" s="1">
+        <v>437</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1499</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="10">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="1">
+        <v>314</v>
+      </c>
+      <c r="E4" s="1">
+        <v>397</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1081</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="10">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="1">
+        <v>318</v>
+      </c>
+      <c r="E5" s="1">
+        <v>387</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1021</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="10">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="1">
+        <v>261</v>
+      </c>
+      <c r="E6" s="1">
+        <v>361</v>
+      </c>
+      <c r="F6" s="1">
+        <v>999</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="10">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1">
+        <v>239</v>
+      </c>
+      <c r="E7" s="1">
+        <v>287</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1099</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="10">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="1">
+        <v>345</v>
+      </c>
+      <c r="E8" s="1">
+        <v>401</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1299</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="10">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="1">
+        <v>261</v>
+      </c>
+      <c r="E9" s="1">
+        <v>291</v>
+      </c>
+      <c r="F9" s="1">
+        <v>999</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="1">
+        <v>303</v>
+      </c>
+      <c r="E10" s="1">
+        <v>387</v>
+      </c>
+      <c r="F10" s="1">
+        <v>899</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="10">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="1">
+        <v>407</v>
+      </c>
+      <c r="E11" s="1">
+        <v>493</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1299</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="10">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="11"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="10">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="11"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="10">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="11"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="10">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="11"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="10">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="11"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="10">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="11"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="10">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="11"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="10">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="11"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="10">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="11"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="10">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="11"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="10">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="11"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="10">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="11"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="10">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="11"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="10">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="11"/>
+    </row>
+    <row r="26" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="12">
+        <v>25</v>
+      </c>
+      <c r="B26" s="13"/>
+      <c r="C26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="14"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{E8AA9AF1-7F06-4857-8FE5-660212E478EE}"/>
+    <hyperlink ref="H4" r:id="rId2" xr:uid="{4665BFA1-22DC-44D9-87A2-5EF59F4E2171}"/>
+    <hyperlink ref="H3" r:id="rId3" xr:uid="{F63491BF-3CC6-4C69-9B6A-C9EEB700FAE3}"/>
+    <hyperlink ref="H5" r:id="rId4" xr:uid="{183B5B8A-7FBC-410A-A3BA-1100283F3C15}"/>
+    <hyperlink ref="H6" r:id="rId5" xr:uid="{3FBA1FA5-ECE3-4147-B3F5-B23A948ECFC5}"/>
+    <hyperlink ref="H7" r:id="rId6" xr:uid="{44FC387D-CE0A-4321-BFE1-7A6042B8ABA2}"/>
+    <hyperlink ref="H8" r:id="rId7" xr:uid="{652C3AF8-7E06-4EDA-955B-10A716DDFD85}"/>
+    <hyperlink ref="H9" r:id="rId8" xr:uid="{A1E17720-194A-4933-BD03-7F2C016B761A}"/>
+    <hyperlink ref="H10" r:id="rId9" xr:uid="{1AB3D33C-C649-4EF3-B46C-0D4C21E27526}"/>
+    <hyperlink ref="H11" r:id="rId10" xr:uid="{A707852E-BD55-4B9E-BF62-24B316824410}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>